<commit_message>
Validar clínicamente las imágenes XAI 101-150
</commit_message>
<xml_diff>
--- a/XAI/muestra-validacion-clinica/muestra_validacion_clinica_150.xlsx
+++ b/XAI/muestra-validacion-clinica/muestra_validacion_clinica_150.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yeray\Desktop\UNIR\Semestre 2\TFM\TFM-UNIR\XAI\muestra-validacion-clinica\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhuar\Desktop\ProyectosIA\TFM\TFM-UNIR\XAI\muestra-validacion-clinica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0DD62C8-9C9C-47DE-8CEA-3F17A5F79D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523664E6-69CA-47E8-96FF-310F1B1B7DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4785" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Etiquetado" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="20">
   <si>
     <t>Número</t>
   </si>
@@ -591,13 +591,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B151"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="28.05" customHeight="1">
+    <row r="1" spans="1:2" ht="28" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1309,301 +1309,401 @@
       <c r="A102" s="5">
         <v>101</v>
       </c>
-      <c r="B102" s="6"/>
+      <c r="B102" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="103" spans="1:2" ht="21" customHeight="1">
       <c r="A103" s="5">
         <v>102</v>
       </c>
-      <c r="B103" s="6"/>
+      <c r="B103" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="104" spans="1:2" ht="21" customHeight="1">
       <c r="A104" s="5">
         <v>103</v>
       </c>
-      <c r="B104" s="6"/>
+      <c r="B104" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="105" spans="1:2" ht="21" customHeight="1">
       <c r="A105" s="5">
         <v>104</v>
       </c>
-      <c r="B105" s="6"/>
+      <c r="B105" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="106" spans="1:2" ht="21" customHeight="1">
       <c r="A106" s="5">
         <v>105</v>
       </c>
-      <c r="B106" s="6"/>
+      <c r="B106" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="107" spans="1:2" ht="21" customHeight="1">
       <c r="A107" s="5">
         <v>106</v>
       </c>
-      <c r="B107" s="6"/>
+      <c r="B107" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="108" spans="1:2" ht="21" customHeight="1">
       <c r="A108" s="5">
         <v>107</v>
       </c>
-      <c r="B108" s="6"/>
+      <c r="B108" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="109" spans="1:2" ht="21" customHeight="1">
       <c r="A109" s="5">
         <v>108</v>
       </c>
-      <c r="B109" s="6"/>
+      <c r="B109" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="110" spans="1:2" ht="21" customHeight="1">
       <c r="A110" s="5">
         <v>109</v>
       </c>
-      <c r="B110" s="6"/>
+      <c r="B110" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="111" spans="1:2" ht="21" customHeight="1">
       <c r="A111" s="5">
         <v>110</v>
       </c>
-      <c r="B111" s="6"/>
+      <c r="B111" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="112" spans="1:2" ht="21" customHeight="1">
       <c r="A112" s="5">
         <v>111</v>
       </c>
-      <c r="B112" s="6"/>
+      <c r="B112" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="113" spans="1:2" ht="21" customHeight="1">
       <c r="A113" s="5">
         <v>112</v>
       </c>
-      <c r="B113" s="6"/>
+      <c r="B113" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="114" spans="1:2" ht="21" customHeight="1">
       <c r="A114" s="5">
         <v>113</v>
       </c>
-      <c r="B114" s="6"/>
+      <c r="B114" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="115" spans="1:2" ht="21" customHeight="1">
       <c r="A115" s="5">
         <v>114</v>
       </c>
-      <c r="B115" s="6"/>
+      <c r="B115" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="116" spans="1:2" ht="21" customHeight="1">
       <c r="A116" s="5">
         <v>115</v>
       </c>
-      <c r="B116" s="6"/>
+      <c r="B116" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="117" spans="1:2" ht="21" customHeight="1">
       <c r="A117" s="5">
         <v>116</v>
       </c>
-      <c r="B117" s="6"/>
+      <c r="B117" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="118" spans="1:2" ht="21" customHeight="1">
       <c r="A118" s="5">
         <v>117</v>
       </c>
-      <c r="B118" s="6"/>
+      <c r="B118" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="119" spans="1:2" ht="21" customHeight="1">
       <c r="A119" s="5">
         <v>118</v>
       </c>
-      <c r="B119" s="6"/>
+      <c r="B119" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="120" spans="1:2" ht="21" customHeight="1">
       <c r="A120" s="5">
         <v>119</v>
       </c>
-      <c r="B120" s="6"/>
+      <c r="B120" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="121" spans="1:2" ht="21" customHeight="1">
       <c r="A121" s="5">
         <v>120</v>
       </c>
-      <c r="B121" s="6"/>
+      <c r="B121" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="122" spans="1:2" ht="21" customHeight="1">
       <c r="A122" s="5">
         <v>121</v>
       </c>
-      <c r="B122" s="6"/>
+      <c r="B122" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="123" spans="1:2" ht="21" customHeight="1">
       <c r="A123" s="5">
         <v>122</v>
       </c>
-      <c r="B123" s="6"/>
+      <c r="B123" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="124" spans="1:2" ht="21" customHeight="1">
       <c r="A124" s="5">
         <v>123</v>
       </c>
-      <c r="B124" s="6"/>
+      <c r="B124" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="125" spans="1:2" ht="21" customHeight="1">
       <c r="A125" s="5">
         <v>124</v>
       </c>
-      <c r="B125" s="6"/>
+      <c r="B125" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="126" spans="1:2" ht="21" customHeight="1">
       <c r="A126" s="5">
         <v>125</v>
       </c>
-      <c r="B126" s="6"/>
+      <c r="B126" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="127" spans="1:2" ht="21" customHeight="1">
       <c r="A127" s="5">
         <v>126</v>
       </c>
-      <c r="B127" s="6"/>
+      <c r="B127" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="128" spans="1:2" ht="21" customHeight="1">
       <c r="A128" s="5">
         <v>127</v>
       </c>
-      <c r="B128" s="6"/>
+      <c r="B128" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="129" spans="1:2" ht="21" customHeight="1">
       <c r="A129" s="5">
         <v>128</v>
       </c>
-      <c r="B129" s="6"/>
+      <c r="B129" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="130" spans="1:2" ht="21" customHeight="1">
       <c r="A130" s="5">
         <v>129</v>
       </c>
-      <c r="B130" s="6"/>
+      <c r="B130" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="131" spans="1:2" ht="21" customHeight="1">
       <c r="A131" s="5">
         <v>130</v>
       </c>
-      <c r="B131" s="6"/>
+      <c r="B131" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="132" spans="1:2" ht="21" customHeight="1">
       <c r="A132" s="5">
         <v>131</v>
       </c>
-      <c r="B132" s="6"/>
+      <c r="B132" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="133" spans="1:2" ht="21" customHeight="1">
       <c r="A133" s="5">
         <v>132</v>
       </c>
-      <c r="B133" s="6"/>
+      <c r="B133" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="134" spans="1:2" ht="21" customHeight="1">
       <c r="A134" s="5">
         <v>133</v>
       </c>
-      <c r="B134" s="6"/>
+      <c r="B134" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="135" spans="1:2" ht="21" customHeight="1">
       <c r="A135" s="5">
         <v>134</v>
       </c>
-      <c r="B135" s="6"/>
+      <c r="B135" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="136" spans="1:2" ht="21" customHeight="1">
       <c r="A136" s="5">
         <v>135</v>
       </c>
-      <c r="B136" s="6"/>
+      <c r="B136" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="137" spans="1:2" ht="21" customHeight="1">
       <c r="A137" s="5">
         <v>136</v>
       </c>
-      <c r="B137" s="6"/>
+      <c r="B137" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="138" spans="1:2" ht="21" customHeight="1">
       <c r="A138" s="5">
         <v>137</v>
       </c>
-      <c r="B138" s="6"/>
+      <c r="B138" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="139" spans="1:2" ht="21" customHeight="1">
       <c r="A139" s="5">
         <v>138</v>
       </c>
-      <c r="B139" s="6"/>
+      <c r="B139" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="140" spans="1:2" ht="21" customHeight="1">
       <c r="A140" s="5">
         <v>139</v>
       </c>
-      <c r="B140" s="6"/>
+      <c r="B140" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="141" spans="1:2" ht="21" customHeight="1">
       <c r="A141" s="5">
         <v>140</v>
       </c>
-      <c r="B141" s="6"/>
+      <c r="B141" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="142" spans="1:2" ht="21" customHeight="1">
       <c r="A142" s="5">
         <v>141</v>
       </c>
-      <c r="B142" s="6"/>
+      <c r="B142" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="143" spans="1:2" ht="21" customHeight="1">
       <c r="A143" s="5">
         <v>142</v>
       </c>
-      <c r="B143" s="6"/>
+      <c r="B143" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="144" spans="1:2" ht="21" customHeight="1">
       <c r="A144" s="5">
         <v>143</v>
       </c>
-      <c r="B144" s="6"/>
+      <c r="B144" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="145" spans="1:2" ht="21" customHeight="1">
       <c r="A145" s="5">
         <v>144</v>
       </c>
-      <c r="B145" s="6"/>
+      <c r="B145" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="146" spans="1:2" ht="21" customHeight="1">
       <c r="A146" s="5">
         <v>145</v>
       </c>
-      <c r="B146" s="6"/>
+      <c r="B146" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="147" spans="1:2" ht="21" customHeight="1">
       <c r="A147" s="5">
         <v>146</v>
       </c>
-      <c r="B147" s="6"/>
+      <c r="B147" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="148" spans="1:2" ht="21" customHeight="1">
       <c r="A148" s="5">
         <v>147</v>
       </c>
-      <c r="B148" s="6"/>
+      <c r="B148" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="149" spans="1:2" ht="21" customHeight="1">
       <c r="A149" s="5">
         <v>148</v>
       </c>
-      <c r="B149" s="6"/>
+      <c r="B149" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="150" spans="1:2" ht="21" customHeight="1">
       <c r="A150" s="5">
         <v>149</v>
       </c>
-      <c r="B150" s="6"/>
+      <c r="B150" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="151" spans="1:2" ht="21" customHeight="1">
       <c r="A151" s="7">
         <v>150</v>
       </c>
-      <c r="B151" s="8"/>
+      <c r="B151" s="8" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B151">
@@ -1623,7 +1723,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1634,7 +1734,7 @@
     <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="31.95" customHeight="1">
+    <row r="1" spans="1:7" ht="32" customHeight="1">
       <c r="A1" s="31" t="s">
         <v>2</v>
       </c>
@@ -1674,7 +1774,7 @@
       </c>
       <c r="G3" s="24">
         <f>COUNTIF(Etiquetado!$B$2:$B$151,"&lt;&gt;")</f>
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1683,22 +1783,22 @@
       </c>
       <c r="B4" s="11">
         <f>COUNTIF(Etiquetado!$B$2:$B$151,A4)</f>
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="C4" s="12">
         <f>B4/$G$2</f>
-        <v>0.08</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="D4" s="13">
         <f>IF($G$3=0,0,B4/$G$3)</f>
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="F4" s="29" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="24">
         <f>G2-G3</f>
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1707,22 +1807,22 @@
       </c>
       <c r="B5" s="15">
         <f>COUNTIF(Etiquetado!$B$2:$B$151,A5)</f>
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="C5" s="16">
         <f>B5/$G$2</f>
-        <v>0.12666666666666668</v>
+        <v>0.24</v>
       </c>
       <c r="D5" s="17">
         <f>IF($G$3=0,0,B5/$G$3)</f>
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="F5" s="29" t="s">
         <v>14</v>
       </c>
       <c r="G5" s="25">
         <f>G3/G2</f>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1731,22 +1831,22 @@
       </c>
       <c r="B6" s="19">
         <f>COUNTIF(Etiquetado!$B$2:$B$151,A6)</f>
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C6" s="20">
         <f>B6/$G$2</f>
-        <v>0.12666666666666668</v>
+        <v>0.26</v>
       </c>
       <c r="D6" s="21">
         <f>IF($G$3=0,0,B6/$G$3)</f>
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="F6" s="29" t="s">
         <v>16</v>
       </c>
       <c r="G6" s="26">
         <f>SUM(B4:B6)</f>
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1755,7 +1855,7 @@
       </c>
       <c r="G7" s="26">
         <f>AVERAGE(B4:B6)</f>
-        <v>16.666666666666668</v>
+        <v>33.333333333333336</v>
       </c>
     </row>
     <row r="8" spans="1:7">

</xml_diff>